<commit_message>
Half-day bell: registry rows, src/day-types.txt date overrides, per-screen 'Bell today' switch
- Bell tab: Half Day (pep-assembly) schedule, periods 0-6 + PR 9:21-10:15
- compile.py: src/day-types.txt lines (DATE  DAY TYPE  note) become exact-date
  day types that win over the DayTypes tab and the weekday rule; unknown types flagged
- room.html: Screen controls > Bell today picks any bell for this screen until
  midnight (sessionStorage), badge shown; all-screens route stays day-types.txt
- docs

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UU6f5Jqpq6x6whEce4kqXF
</commit_message>
<xml_diff>
--- a/src/registry/EHS_room_display_data.xlsx
+++ b/src/registry/EHS_room_display_data.xlsx
@@ -1528,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1542,7 +1542,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Real EHS bell, 2025-26 pattern (unchanged for 2026-27). Regular = Mon/Tue/Thu/Fri; Wednesday = every Wednesday (wired in DayTypes). Lunch waves A-D run inside 4th hour (Regular) and 5th hour (Wednesday); the display treats those as one long period. Times accept 7:15 AM style.</t>
+          <t>Real EHS bell, 2025-26 pattern (unchanged for 2026-27). Regular = Mon/Tue/Thu/Fri; Wednesday = every Wednesday (wired in DayTypes). Lunch waves A-D run inside 4th hour (Regular) and 5th hour (Wednesday); the display treats those as one long period. Times accept 7:15 AM style. Half Day = the 1/2-day pep-assembly bell (15-minute periods, pep rally 9:21-10:15); schedule it for a date in src/day-types.txt or the DayTypes tab, or pick it on a screen under Screen controls &gt; Bell.</t>
         </is>
       </c>
     </row>
@@ -1977,6 +1977,238 @@
         </is>
       </c>
       <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Zero Hour</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>6:25 AM</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>7:10 AM</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Early bird</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>1st Hour</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>7:15 AM</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>7:30 AM</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>2nd Hour</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>7:36 AM</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>7:51 AM</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>3rd Hour</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>7:57 AM</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>8:12 AM</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>4th Hour</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>8:18 AM</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>8:33 AM</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>5th Hour</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>8:39 AM</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>8:54 AM</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>6th Hour</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>9:15 AM</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Half Day</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Pep Rally</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>9:21 AM</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>10:15 AM</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>No course is mapped to PR, so every screen shows announcements</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2003,7 +2235,7 @@
     <row r="1" ht="44" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Exact-date rows override everything; a weekday name (Wednesday) applies every week. A day type with no Bell rows = announcements only, all day. No-school dates below are the 2026-27 district calendar. NOTE: the three half days (Aug 19, Oct 23, May 25) are NOT listed - they run the normal bell. Add them with a Half Day bell once those times are published.</t>
+          <t>Exact-date rows override everything; a weekday name (Wednesday) applies every week. A day type with no Bell rows = announcements only, all day. No-school dates below are the 2026-27 district calendar. Half days: a 'Half Day' bell now exists - add a row here (date -&gt; Half Day) or, easier from a phone, a line in src/day-types.txt.</t>
         </is>
       </c>
     </row>

</xml_diff>